<commit_message>
fix all collages placement data
</commit_message>
<xml_diff>
--- a/exports/colleges/25446_all-india-institute-of-medical-sciences-aiims-new-delhi.xlsx
+++ b/exports/colleges/25446_all-india-institute-of-medical-sciences-aiims-new-delhi.xlsx
@@ -593,18 +593,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="75" customWidth="1" min="3" max="3"/>
-    <col width="75" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="3" max="3"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="39" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
@@ -685,12 +685,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Master of Science [M.Sc] (Clinical Embryology and Reproductive Biology)</t>
+          <t>Master of Science [M.Sc]</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Master of Science [M.Sc] (Clinical Embryology and Reproductive Biology)</t>
+          <t>Master of Science [M.Sc]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -710,12 +710,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Graduation</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>AIIMS MSc</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>10+2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>AIIMS Paramedical, AIIMS BSc Nursing</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -809,12 +809,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Bachelor of Science [B.Sc] (Medical Radiology \u0026 Imaging Technology)</t>
+          <t>Bachelor of Science [B.Sc]</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bachelor of Science [B.Sc] (Medical Radiology \u0026 Imaging Technology)</t>
+          <t>Bachelor of Science [B.Sc]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>3 Years 6 Months</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -834,12 +834,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>10+2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>AIIMS Paramedical, AIIMS BSc Nursing</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -866,57 +866,119 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>MBBS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Doctor of Medicine [MD] (Medicine)</t>
+          <t>M.B.B.S.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Doctor of Medicine [MD] (Medicine)</t>
+          <t>M.B.B.S.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>5,356</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>5 Years 6 Months</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>10+2 + NEET</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>NEET</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MDS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Master of Dental Surgery [MDS]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Master of Dental Surgery [MDS]</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>7,577</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>Full Time</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>UG</t>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>B.D.S. with 55% + INI-CET</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>INI CET</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1068,17 +1130,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>67.80 LPA</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>16 LPA</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>13.5 Lakh</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">

</xml_diff>

<commit_message>
placement and ranking issue fix
</commit_message>
<xml_diff>
--- a/exports/colleges/25446_all-india-institute-of-medical-sciences-aiims-new-delhi.xlsx
+++ b/exports/colleges/25446_all-india-institute-of-medical-sciences-aiims-new-delhi.xlsx
@@ -25,13 +25,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,72 +453,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>college_type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>ownership</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>established_year</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>accreditation</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>affiliation</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>rating</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ranking</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>overview_description</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>contact_info</t>
         </is>
@@ -593,17 +605,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="47" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
     <col width="39" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
@@ -611,62 +623,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>degree_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>course_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>specialization</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>total_fees</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>duration</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>course_type</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>eligibility</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>entrance_exam</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>application_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>intake_seats</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>course_level</t>
         </is>
@@ -710,7 +722,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Graduation</t>
+          <t>Graduation with 60%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -866,27 +878,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MBBS</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>M.B.B.S.</t>
+          <t>Doctor of Medicine [MD]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>M.B.B.S.</t>
+          <t>Doctor of Medicine [MD]</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>5,356</t>
+          <t>7,577</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5 Years 6 Months</t>
+          <t>3 Years</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -896,12 +908,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>10+2 + NEET</t>
+          <t>MBBS with 55% + INI-CET</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NEET</t>
+          <t>INI SS, INI CET</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -916,7 +928,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -928,55 +940,3073 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>M.B.B.S.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>M.B.B.S.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5,356</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>5 Years 6 Months</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>10+2 + NEET</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NEET</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B.Sc {Hons.}</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>B.Sc {Hons.}</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2,965 - 39,095</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2,970 - 4,480</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2,830 - 7,577</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>NEET PG</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>5,356</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5 Years 6 Months</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NEET</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>12,125</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3-5 Years</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>GATE / UGC NET</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>MDS</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Master of Dental Surgery [MDS]</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Master of Dental Surgery [MDS]</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MDS</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MDS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>7,577</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>3 Years</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Full Time</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>B.D.S. with 55% + INI-CET</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>INI CET</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>NEET PG</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>6,050</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>M.Ch</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>M.Ch</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>M.Ch</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>6,050</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Clinical Embryology and Reproductive Biology</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Clinical Embryology and Reproductive Biology</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Nursing</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Nursing</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nuclear Medicine Technology</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Nuclear Medicine Technology</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Medical Pharmacology</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medical Pharmacology</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Medical Anatomy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medical Anatomy</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Medical Physiology</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Medical Physiology</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Biophysics</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Biophysics</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Nephrology Nursing</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Nephrology Nursing</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Neuroscience Nursing</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Neuroscience Nursing</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Critical Care Nursing</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Critical Care Nursing</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Psychiatric Nursing</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Psychiatric Nursing</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Cardiological / CTVS Nursing</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Cardiological / CTVS Nursing</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Oncology Nursing</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Oncology Nursing</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Paediatric Nursing</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Paediatric Nursing</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Perfusion Technology</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Perfusion Technology</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2,830</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>B.Sc {Hons.} Nursing</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>B.Sc {Hons.} Nursing</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>39,095</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>B.Sc Medical Radiology &amp; Imaging Technology</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>B.Sc Medical Radiology &amp; Imaging Technology</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>4,480</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>B.Sc Operation Theatre Technology</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>B.Sc Operation Theatre Technology</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>3,385</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>B.Sc Dental Hygiene</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>B.Sc Dental Hygiene</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>3,385</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>B.Sc Dental Operating Room Assistant</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>B.Sc Dental Operating Room Assistant</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>3,385</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MD (General)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2,830 - 7,577</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MBBS (General)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>5,356</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ph.D (General)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>12,125</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>3-5 Years</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>GATE / UGC NET</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>3.4 Lakhs</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>3-5 Years</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Postgraduation in relevant field</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>GATE / UGC NET</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>3.4 Lakhs</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>3-5 Years</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Postgraduation in relevant field</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>GATE / UGC NET</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Humanities And Social Science</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Humanities And Social Science</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>3.4 Lakhs</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>3-5 Years</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Postgraduation in relevant field</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>GATE / UGC NET</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Public Policy</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Public Policy</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>3.4 Lakhs</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>3-5 Years</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Postgraduation in relevant field</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>GATE / UGC NET</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MDS</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MDS (General)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>7,577</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>DM (General)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>6,050</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>M.Ch</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>M.Ch (General)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>6,050</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Exam Frequency</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Exam Frequency</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Exam Frequency</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Once a year</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Mode of Examination</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Mode of Examination</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Mode of Examination</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Computer-Based Test (CBT)/Online</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Courses Offered</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Courses Offered</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Courses Offered</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>BSc (Hons.) Nursing and BSc (Post-Basic) Nursing</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Seats Offered</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Seats Offered</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Seats Offered</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BSc Nursing (Post-Basic)- 20 BSc Nursing (Hons.)- 571</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Exam Fee</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Exam Fee</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Exam Fee</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>General and OBC: 1,500 SC, ST and EWS: 1,200 PwBD: Nil</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Language of the Exam</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Language of the Exam</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Language of the Exam</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Exam Duration</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Exam Duration</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Exam Duration</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Two hours</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Total Marks</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Total Marks</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Total Marks</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Total Questions</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Total Questions</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Total Questions</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>25446</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Marking Scheme</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Marking Scheme</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>+1 for each correct answer -1/3 for each incorrect answer</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
@@ -1005,32 +4035,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>admission_process</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>exams_accepted</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>eligibility_criteria</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>important_dates</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>application_deadlines</t>
         </is>
@@ -1091,32 +4121,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>highest_package</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>average_package</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>median_package</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>placement_percentage</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>top_recruiters</t>
         </is>
@@ -1175,22 +4205,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ranking_body</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ranking_year</t>
         </is>
@@ -1233,12 +4263,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1275,12 +4305,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1318,17 +4348,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>hostel_fees</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>facilities</t>
         </is>
@@ -1366,28 +4396,28 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="552" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>college_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>reviewer_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>rating</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>review_text</t>
         </is>
@@ -1401,7 +4431,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aditya Sharma</t>
+          <t>Alumni Reviewer</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1409,7 +4439,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Excellent academic atmosphere, world class research facilities, and amazing placements.</t>
+          <t>Pros: While measuring the faculty-to-student ratio, it is evident that both the faculty and the student population fall within a desirable range. All the professors here have either completed postgraduate studies or obtained a masters degree in their respective fields. Interns are posted in OPDs, wards, labs, etc., gaining valuable clinical exposure and experience. The placement scenario here is very good, with about 80% or more in various drug agencies and hospitals. The average salary offered is about 7-9 LPA, which is a really good package.</t>
         </is>
       </c>
     </row>

</xml_diff>